<commit_message>
Daily recap, matchup updates, learning and research 2026-08-17
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-17.xlsx
+++ b/data/k-props/2026-08-17.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="85">
   <si>
     <t>date</t>
   </si>
@@ -145,19 +145,31 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Rhett Lowder</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Brandon Young</t>
+  </si>
+  <si>
+    <t>Baltimore Orioles @ Tampa Bay Rays</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Rhett Lowder</t>
-  </si>
-  <si>
-    <t>Brandon Young</t>
-  </si>
-  <si>
-    <t>Baltimore Orioles @ Tampa Bay Rays</t>
   </si>
   <si>
     <t>Shane McClanahan</t>
@@ -835,17 +847,23 @@
       <c r="Y2">
         <v>1.068</v>
       </c>
+      <c r="Z2">
+        <v>5</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>0.88</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>5.22</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.1713</v>
@@ -855,6 +873,18 @@
       </c>
       <c r="AH2">
         <v>0.16</v>
+      </c>
+      <c r="AI2">
+        <v>-0.22</v>
+      </c>
+      <c r="AJ2">
+        <v>0.22</v>
+      </c>
+      <c r="AK2">
+        <v>-0.38</v>
+      </c>
+      <c r="AL2">
+        <v>0.38</v>
       </c>
       <c r="AM2">
         <v>5.38</v>
@@ -865,7 +895,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -936,17 +966,23 @@
       <c r="Y3">
         <v>0.9246</v>
       </c>
+      <c r="Z3">
+        <v>5</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>-1.1</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>3.24</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.1778</v>
@@ -956,6 +992,18 @@
       </c>
       <c r="AH3">
         <v>0.16</v>
+      </c>
+      <c r="AI3">
+        <v>1.76</v>
+      </c>
+      <c r="AJ3">
+        <v>1.76</v>
+      </c>
+      <c r="AK3">
+        <v>1.6</v>
+      </c>
+      <c r="AL3">
+        <v>1.6</v>
       </c>
       <c r="AM3">
         <v>3.4</v>
@@ -966,7 +1014,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>3.5</v>
@@ -978,7 +1026,7 @@
         <v>115</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>822939</v>
@@ -1037,17 +1085,23 @@
       <c r="Y4">
         <v>0.88</v>
       </c>
+      <c r="Z4">
+        <v>3</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB4">
+        <v>0.08</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD4">
         <v>3.42</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.1981</v>
@@ -1057,6 +1111,18 @@
       </c>
       <c r="AH4">
         <v>0.16</v>
+      </c>
+      <c r="AI4">
+        <v>-0.42</v>
+      </c>
+      <c r="AJ4">
+        <v>0.42</v>
+      </c>
+      <c r="AK4">
+        <v>-0.58</v>
+      </c>
+      <c r="AL4">
+        <v>0.58</v>
       </c>
       <c r="AM4">
         <v>3.58</v>
@@ -1067,7 +1133,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1079,7 +1145,7 @@
         <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>822939</v>
@@ -1138,17 +1204,23 @@
       <c r="Y5">
         <v>1.0638</v>
       </c>
+      <c r="Z5">
+        <v>3</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB5">
+        <v>0.94</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD5">
         <v>5.28</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.2104</v>
@@ -1158,6 +1230,18 @@
       </c>
       <c r="AH5">
         <v>0.16</v>
+      </c>
+      <c r="AI5">
+        <v>-2.28</v>
+      </c>
+      <c r="AJ5">
+        <v>2.28</v>
+      </c>
+      <c r="AK5">
+        <v>-2.44</v>
+      </c>
+      <c r="AL5">
+        <v>2.44</v>
       </c>
       <c r="AM5">
         <v>5.44</v>
@@ -1168,7 +1252,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C6">
         <v>3.5</v>
@@ -1180,7 +1264,7 @@
         <v>-155</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>823427</v>
@@ -1239,17 +1323,23 @@
       <c r="Y6">
         <v>0.9355</v>
       </c>
+      <c r="Z6">
+        <v>2</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB6">
+        <v>-0.54</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD6">
         <v>2.8</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.1694</v>
@@ -1259,6 +1349,18 @@
       </c>
       <c r="AH6">
         <v>0.16</v>
+      </c>
+      <c r="AI6">
+        <v>-0.8</v>
+      </c>
+      <c r="AJ6">
+        <v>0.8</v>
+      </c>
+      <c r="AK6">
+        <v>-0.96</v>
+      </c>
+      <c r="AL6">
+        <v>0.96</v>
       </c>
       <c r="AM6">
         <v>2.96</v>
@@ -1269,10 +1371,10 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>823427</v>
@@ -1332,16 +1434,16 @@
         <v>1.0099</v>
       </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD7">
         <v>8.29</v>
       </c>
       <c r="AE7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="AF7">
         <v>0.2898</v>
@@ -1361,7 +1463,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>5.5</v>
@@ -1373,7 +1475,7 @@
         <v>-143</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G8">
         <v>823343</v>
@@ -1432,17 +1534,23 @@
       <c r="Y8">
         <v>1.1071</v>
       </c>
+      <c r="Z8">
+        <v>5</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB8">
+        <v>0.2</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD8">
         <v>5.54</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.1733</v>
@@ -1452,6 +1560,18 @@
       </c>
       <c r="AH8">
         <v>0.16</v>
+      </c>
+      <c r="AI8">
+        <v>-0.54</v>
+      </c>
+      <c r="AJ8">
+        <v>0.54</v>
+      </c>
+      <c r="AK8">
+        <v>-0.7</v>
+      </c>
+      <c r="AL8">
+        <v>0.7</v>
       </c>
       <c r="AM8">
         <v>5.7</v>
@@ -1462,7 +1582,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>2.5</v>
@@ -1474,13 +1594,13 @@
         <v>133</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>823343</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I9">
         <v>4.5</v>
@@ -1533,17 +1653,23 @@
       <c r="Y9">
         <v>0.88</v>
       </c>
+      <c r="Z9">
+        <v>3</v>
+      </c>
       <c r="AA9" t="s">
         <v>44</v>
       </c>
+      <c r="AB9">
+        <v>0.22</v>
+      </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD9">
         <v>2.56</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.1531</v>
@@ -1553,6 +1679,18 @@
       </c>
       <c r="AH9">
         <v>0.16</v>
+      </c>
+      <c r="AI9">
+        <v>0.44</v>
+      </c>
+      <c r="AJ9">
+        <v>0.44</v>
+      </c>
+      <c r="AK9">
+        <v>0.28</v>
+      </c>
+      <c r="AL9">
+        <v>0.28</v>
       </c>
       <c r="AM9">
         <v>2.72</v>
@@ -1563,7 +1701,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C10">
         <v>3.5</v>
@@ -1575,7 +1713,7 @@
         <v>114</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <v>824725</v>
@@ -1634,17 +1772,23 @@
       <c r="Y10">
         <v>0.9787</v>
       </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB10">
+        <v>0.26</v>
       </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD10">
         <v>3.6</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.1808</v>
@@ -1654,6 +1798,18 @@
       </c>
       <c r="AH10">
         <v>0.16</v>
+      </c>
+      <c r="AI10">
+        <v>-3.6</v>
+      </c>
+      <c r="AJ10">
+        <v>3.6</v>
+      </c>
+      <c r="AK10">
+        <v>-3.76</v>
+      </c>
+      <c r="AL10">
+        <v>3.76</v>
       </c>
       <c r="AM10">
         <v>3.76</v>
@@ -1664,16 +1820,16 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G11">
         <v>824725</v>
       </c>
       <c r="H11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I11">
         <v>4.5</v>
@@ -1694,7 +1850,7 @@
         <v>4</v>
       </c>
       <c r="S11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="T11">
         <v>0.1775</v>
@@ -1715,16 +1871,16 @@
         <v>0.912</v>
       </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD11">
         <v>2.3</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.1765</v>
@@ -1744,7 +1900,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>3.5</v>
@@ -1756,7 +1912,7 @@
         <v>125</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12">
         <v>823589</v>
@@ -1815,17 +1971,23 @@
       <c r="Y12">
         <v>0.9654</v>
       </c>
+      <c r="Z12">
+        <v>4</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>1.15</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
         <v>4.49</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.1917</v>
@@ -1835,6 +1997,18 @@
       </c>
       <c r="AH12">
         <v>0.16</v>
+      </c>
+      <c r="AI12">
+        <v>-0.49</v>
+      </c>
+      <c r="AJ12">
+        <v>0.49</v>
+      </c>
+      <c r="AK12">
+        <v>-0.65</v>
+      </c>
+      <c r="AL12">
+        <v>0.65</v>
       </c>
       <c r="AM12">
         <v>4.65</v>
@@ -1845,7 +2019,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C13">
         <v>5.5</v>
@@ -1857,7 +2031,7 @@
         <v>120</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>823589</v>
@@ -1916,17 +2090,23 @@
       <c r="Y13">
         <v>1.0012</v>
       </c>
+      <c r="Z13">
+        <v>3</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB13">
+        <v>-0.17</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD13">
         <v>5.17</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.2812</v>
@@ -1936,6 +2116,18 @@
       </c>
       <c r="AH13">
         <v>0.16</v>
+      </c>
+      <c r="AI13">
+        <v>-2.17</v>
+      </c>
+      <c r="AJ13">
+        <v>2.17</v>
+      </c>
+      <c r="AK13">
+        <v>-2.33</v>
+      </c>
+      <c r="AL13">
+        <v>2.33</v>
       </c>
       <c r="AM13">
         <v>5.33</v>
@@ -1946,7 +2138,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>3.5</v>
@@ -1958,13 +2150,13 @@
         <v>-139</v>
       </c>
       <c r="F14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G14">
         <v>824077</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I14">
         <v>4.4</v>
@@ -2017,17 +2209,23 @@
       <c r="Y14">
         <v>0.9548</v>
       </c>
+      <c r="Z14">
+        <v>2</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB14">
+        <v>0.38</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD14">
         <v>3.72</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.2142</v>
@@ -2037,6 +2235,18 @@
       </c>
       <c r="AH14">
         <v>0.16</v>
+      </c>
+      <c r="AI14">
+        <v>-1.72</v>
+      </c>
+      <c r="AJ14">
+        <v>1.72</v>
+      </c>
+      <c r="AK14">
+        <v>-1.88</v>
+      </c>
+      <c r="AL14">
+        <v>1.88</v>
       </c>
       <c r="AM14">
         <v>3.88</v>
@@ -2047,7 +2257,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2059,7 +2269,7 @@
         <v>-125</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G15">
         <v>824077</v>
@@ -2118,17 +2328,23 @@
       <c r="Y15">
         <v>0.9819</v>
       </c>
+      <c r="Z15">
+        <v>3</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB15">
+        <v>-0.55</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD15">
         <v>3.79</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.1823</v>
@@ -2138,6 +2354,18 @@
       </c>
       <c r="AH15">
         <v>0.16</v>
+      </c>
+      <c r="AI15">
+        <v>-0.79</v>
+      </c>
+      <c r="AJ15">
+        <v>0.79</v>
+      </c>
+      <c r="AK15">
+        <v>-0.95</v>
+      </c>
+      <c r="AL15">
+        <v>0.95</v>
       </c>
       <c r="AM15">
         <v>3.95</v>
@@ -2148,10 +2376,10 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G16">
         <v>823668</v>
@@ -2211,16 +2439,16 @@
         <v>0.9396</v>
       </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD16">
         <v>3.37</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1859</v>
@@ -2240,7 +2468,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C17">
         <v>3.5</v>
@@ -2252,7 +2480,7 @@
         <v>-119</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G17">
         <v>823668</v>
@@ -2311,17 +2539,23 @@
       <c r="Y17">
         <v>0.9357</v>
       </c>
+      <c r="Z17">
+        <v>4</v>
+      </c>
       <c r="AA17" t="s">
         <v>44</v>
       </c>
+      <c r="AB17">
+        <v>-0.17</v>
+      </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD17">
         <v>3.17</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1533</v>
@@ -2331,6 +2565,18 @@
       </c>
       <c r="AH17">
         <v>0.16</v>
+      </c>
+      <c r="AI17">
+        <v>0.83</v>
+      </c>
+      <c r="AJ17">
+        <v>0.83</v>
+      </c>
+      <c r="AK17">
+        <v>0.67</v>
+      </c>
+      <c r="AL17">
+        <v>0.67</v>
       </c>
       <c r="AM17">
         <v>3.33</v>
@@ -2341,7 +2587,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18">
         <v>4.5</v>
@@ -2353,7 +2599,7 @@
         <v>100</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G18">
         <v>824641</v>
@@ -2392,7 +2638,7 @@
         <v>0.373</v>
       </c>
       <c r="S18" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="T18">
         <v>0.2302</v>
@@ -2412,17 +2658,23 @@
       <c r="Y18">
         <v>0.9619</v>
       </c>
+      <c r="Z18">
+        <v>1</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="AB18">
+        <v>0.32</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD18">
         <v>4.66</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
         <v>0.2061</v>
@@ -2432,6 +2684,18 @@
       </c>
       <c r="AH18">
         <v>0.16</v>
+      </c>
+      <c r="AI18">
+        <v>-3.66</v>
+      </c>
+      <c r="AJ18">
+        <v>3.66</v>
+      </c>
+      <c r="AK18">
+        <v>-3.82</v>
+      </c>
+      <c r="AL18">
+        <v>3.82</v>
       </c>
       <c r="AM18">
         <v>4.82</v>
@@ -2442,7 +2706,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C19">
         <v>5.5</v>
@@ -2454,7 +2718,7 @@
         <v>110</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>824641</v>
@@ -2513,17 +2777,23 @@
       <c r="Y19">
         <v>0.9688</v>
       </c>
+      <c r="Z19">
+        <v>10</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-0.04</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD19">
         <v>5.3</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.2276</v>
@@ -2533,6 +2803,18 @@
       </c>
       <c r="AH19">
         <v>0.16</v>
+      </c>
+      <c r="AI19">
+        <v>4.7</v>
+      </c>
+      <c r="AJ19">
+        <v>4.7</v>
+      </c>
+      <c r="AK19">
+        <v>4.54</v>
+      </c>
+      <c r="AL19">
+        <v>4.54</v>
       </c>
       <c r="AM19">
         <v>5.46</v>
@@ -2543,7 +2825,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>2.5</v>
@@ -2555,7 +2837,7 @@
         <v>136</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>824320</v>
@@ -2614,17 +2896,23 @@
       <c r="Y20">
         <v>0.9901</v>
       </c>
+      <c r="Z20">
+        <v>3</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>0.61</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD20">
         <v>2.95</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.1451</v>
@@ -2634,6 +2922,18 @@
       </c>
       <c r="AH20">
         <v>0.16</v>
+      </c>
+      <c r="AI20">
+        <v>0.05</v>
+      </c>
+      <c r="AJ20">
+        <v>0.05</v>
+      </c>
+      <c r="AK20">
+        <v>-0.11</v>
+      </c>
+      <c r="AL20">
+        <v>0.11</v>
       </c>
       <c r="AM20">
         <v>3.11</v>
@@ -2644,7 +2944,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21">
         <v>4.5</v>
@@ -2659,28 +2959,28 @@
         <v>41</v>
       </c>
       <c r="G21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L21">
         <v>6</v>
       </c>
       <c r="S21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE21" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:39" x14ac:dyDescent="0.25">
@@ -2688,7 +2988,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C22">
         <v>6.5</v>
@@ -2700,31 +3000,31 @@
         <v>108</v>
       </c>
       <c r="F22" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L22">
         <v>6</v>
       </c>
       <c r="S22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:39" x14ac:dyDescent="0.25">
@@ -2732,7 +3032,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C23">
         <v>3.5</v>
@@ -2744,31 +3044,31 @@
         <v>-109</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L23">
         <v>6</v>
       </c>
       <c r="S23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE23" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:39" x14ac:dyDescent="0.25">
@@ -2776,7 +3076,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C24">
         <v>6.5</v>
@@ -2788,31 +3088,34 @@
         <v>117</v>
       </c>
       <c r="F24" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G24" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H24" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L24">
         <v>6</v>
       </c>
       <c r="S24" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V24" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="Z24">
+        <v>5</v>
       </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE24" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>